<commit_message>
resolved conflicts and completed 5+4 scenarios
</commit_message>
<xml_diff>
--- a/src/main/resources/UserRegistration_Field_Values.xlsx
+++ b/src/main/resources/UserRegistration_Field_Values.xlsx
@@ -8,30 +8,31 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workpace-gov-grants-framework-automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F01A98F5-C369-4BC9-8F06-3CEFE60A8657}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0D139B8-C64A-468C-B595-A0AD42437487}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CreationWithAllDetails" sheetId="1" r:id="rId1"/>
-    <sheet name="CreationWithOnlyPaymentDetail" sheetId="20" r:id="rId2"/>
-    <sheet name="PrimaryRepresentativeDetails" sheetId="14" r:id="rId3"/>
-    <sheet name="OrgAddressOtherThanUSA" sheetId="13" r:id="rId4"/>
-    <sheet name="CreationQ1NO" sheetId="19" r:id="rId5"/>
-    <sheet name="UniqueOrgInfoQuestionsNoExplain" sheetId="15" r:id="rId6"/>
-    <sheet name="WithQues1YesDetailExplain" sheetId="16" r:id="rId7"/>
-    <sheet name="WithQues1YesNICRAYes" sheetId="17" r:id="rId8"/>
-    <sheet name="WithQues1YesOrgIncorYes" sheetId="18" r:id="rId9"/>
-    <sheet name="Question1" sheetId="2" r:id="rId10"/>
-    <sheet name="Question2" sheetId="4" r:id="rId11"/>
-    <sheet name="Question1No" sheetId="3" r:id="rId12"/>
-    <sheet name="Question2No" sheetId="5" r:id="rId13"/>
-    <sheet name="UniqueOrgInfoQuestions" sheetId="6" r:id="rId14"/>
-    <sheet name="OrgAddress" sheetId="7" r:id="rId15"/>
-    <sheet name="OrgProfile" sheetId="8" r:id="rId16"/>
-    <sheet name="OrgProfileCompleteDetail" sheetId="9" r:id="rId17"/>
-    <sheet name="WithQues1YesAndRelatedDetailsNo" sheetId="11" r:id="rId18"/>
-    <sheet name="WithQues1YesAndRelatedDetailYes" sheetId="12" r:id="rId19"/>
+    <sheet name="OrgRegCreationCompleteDetail" sheetId="21" r:id="rId2"/>
+    <sheet name="CreationWithOnlyPaymentDetail" sheetId="20" r:id="rId3"/>
+    <sheet name="PrimaryRepresentativeDetails" sheetId="14" r:id="rId4"/>
+    <sheet name="OrgAddressOtherThanUSA" sheetId="13" r:id="rId5"/>
+    <sheet name="CreationQ1NO" sheetId="19" r:id="rId6"/>
+    <sheet name="UniqueOrgInfoQuestionsNoExplain" sheetId="15" r:id="rId7"/>
+    <sheet name="WithQues1YesDetailExplain" sheetId="16" r:id="rId8"/>
+    <sheet name="WithQues1YesNICRAYes" sheetId="17" r:id="rId9"/>
+    <sheet name="WithQues1YesOrgIncorYes" sheetId="18" r:id="rId10"/>
+    <sheet name="Question1" sheetId="2" r:id="rId11"/>
+    <sheet name="Question2" sheetId="4" r:id="rId12"/>
+    <sheet name="Question1No" sheetId="3" r:id="rId13"/>
+    <sheet name="Question2No" sheetId="5" r:id="rId14"/>
+    <sheet name="UniqueOrgInfoQuestions" sheetId="6" r:id="rId15"/>
+    <sheet name="OrgAddress" sheetId="7" r:id="rId16"/>
+    <sheet name="OrgProfile" sheetId="8" r:id="rId17"/>
+    <sheet name="OrgProfileCompleteDetail" sheetId="9" r:id="rId18"/>
+    <sheet name="WithQues1YesAndRelatedDetailsNo" sheetId="11" r:id="rId19"/>
+    <sheet name="WithQues1YesAndRelatedDetailYes" sheetId="12" r:id="rId20"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="90">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -937,6 +938,107 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14F6A843-34CB-40B2-914A-08E2C54EB350}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="2" max="2" width="28.46484375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A00A2F9B-1F15-474D-9DD4-993171530508}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -972,7 +1074,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05EFA198-FBA1-4B9A-B3E9-28166FF18612}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -1008,7 +1110,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF1A298F-7844-48D1-98DD-53D7D86DE791}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -1043,7 +1145,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69C6C8DD-009D-425E-9B69-09D5E0ACEE9D}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -1078,7 +1180,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E2F0CAC-30A4-45BD-AE27-07806349BD24}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -1125,7 +1227,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5343F989-BED4-4C3F-AE8F-330830F9208D}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -1220,7 +1322,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B216D1F-84FF-4062-A939-3C635B054F5E}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -1279,7 +1381,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61C7FB28-3C46-41CD-B1C8-5ACD5AA83D43}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -1360,7 +1462,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B080C06C-48BE-4956-AB6C-FA9A46DD80B4}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -1430,7 +1532,168 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{656D3EEC-31AD-4355-BD03-CC983BBF34F9}">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="8.06640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.06640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.1328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="20" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="24" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="24" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="22" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" s="24" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="22" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="22">
+        <v>20171</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="C13" s="22" t="s">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C5" r:id="rId1" xr:uid="{FA019F3C-CAF3-40BA-A6D4-430C2E40DA3F}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44E55028-70E0-4DC2-93F0-398F08D85BA5}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -1511,7 +1774,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9428DC2-E37D-4A86-AEA0-C4AB0CF98F92}">
   <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -1630,7 +1893,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4BF3096-62C1-489E-B677-AEC71181CA96}">
   <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -1778,7 +2041,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BCE78A5-F6A7-4E3D-A256-8FF61363066F}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -1873,7 +2136,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C74A7102-EF70-435E-8D51-B513DF0574A2}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -1968,7 +2231,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B84EBB0-BE12-4675-B5CC-0B8071F9EF1D}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -2022,7 +2285,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6905C96-681E-4E14-B81E-3B11E237FCA3}">
   <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -2120,7 +2383,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1AA2095-5BE4-441A-914C-113834C7CAC4}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -2205,105 +2468,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14F6A843-34CB-40B2-914A-08E2C54EB350}">
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
-  <cols>
-    <col min="2" max="2" width="28.46484375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="12" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" s="13" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" s="13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" s="13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="C5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="C6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="C7" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>